<commit_message>
commit 15 - added more data and analysis
</commit_message>
<xml_diff>
--- a/continous/analysis_continuous.xlsx
+++ b/continous/analysis_continuous.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/calld-admin/Documents/stoix-backup/stoix_snapshot/Stoix/continous/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{20AAAA27-0B22-8646-8C13-476B081668C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F5D5049-6131-5B46-B9C8-BC3B058AD09E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17440" xr2:uid="{D90AB766-58C8-154D-A5F6-94AF14BE3E23}"/>
+    <workbookView xWindow="30240" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{D90AB766-58C8-154D-A5F6-94AF14BE3E23}"/>
   </bookViews>
   <sheets>
     <sheet name="analysis" sheetId="1" r:id="rId1"/>

</xml_diff>